<commit_message>
docs: fuente de costos Costos.xlsx versionada + memory al dia
</commit_message>
<xml_diff>
--- a/assets/docs/Costos.xlsx
+++ b/assets/docs/Costos.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zcoder\Documents\CYCSWeb\GitHub\plan_red-wifi_posada\assets\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2677EEB0-DA04-4214-B6E5-CA44DA635DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Costos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,11 +24,75 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>EQUIPAMIENTO</t>
+  </si>
+  <si>
+    <t>Cantidad</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Precio Unitario ($)</t>
+  </si>
+  <si>
+    <t>Sub-total ($)</t>
+  </si>
+  <si>
+    <t>AP GWN7661</t>
+  </si>
+  <si>
+    <t>Switch GWN7801p</t>
+  </si>
+  <si>
+    <t>Bobina Cable UTP Cat.6e</t>
+  </si>
+  <si>
+    <t>Sub-Total ($)</t>
+  </si>
+  <si>
+    <t>MANO DE OBRA</t>
+  </si>
+  <si>
+    <t>A convenir</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,13 +116,33 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +420,114 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:E15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="D2" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1">
+        <v>139.5</v>
+      </c>
+      <c r="E6" s="1">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1">
+        <v>208.5</v>
+      </c>
+      <c r="E7" s="1">
+        <v>208.5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="1">
+        <v>1</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="1">
+        <v>100</v>
+      </c>
+      <c r="E8" s="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="1"/>
+      <c r="C10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1">
+        <v>587.5</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="D13" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="6">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>